<commit_message>
ensuring hpc time per sim is present
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1D0339-9B8D-4DF3-977A-B78BA3D86285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Summary"/>
+    <sheet name="Summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -97,8 +116,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -121,14 +139,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3f3f76"/>
+      <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3f3f3f"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -142,17 +160,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffffcc"/>
+        <fgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFffcc99"/>
+        <fgColor rgb="FFFFCC99"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFf2f2f2"/>
+        <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -208,7 +226,7 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -241,7 +259,7 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -253,7 +271,7 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -262,7 +280,7 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -277,7 +295,7 @@
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -286,13 +304,13 @@
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -300,116 +318,113 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="24">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="4" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="6" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="7" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="6" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="8" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="9" applyBorder="1" fontId="2" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="9" applyBorder="1" fontId="3" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="10" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:M42" displayName="Table1" name="Table1" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:M42"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M42" totalsRowShown="0">
+  <autoFilter ref="A1:M42" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="13">
-    <tableColumn name="hardware_utilization_strategy" id="1"/>
-    <tableColumn name="device" id="2"/>
-    <tableColumn name="run_mode" id="3"/>
-    <tableColumn name="n_nodes" id="4"/>
-    <tableColumn name="n_mpi_procs" id="5"/>
-    <tableColumn name="n_omp_threads" id="6"/>
-    <tableColumn name="n_gpus" id="7"/>
-    <tableColumn name="hpc_ensemble_partition" id="8"/>
-    <tableColumn name="hpc_time_min_per_sim" id="9"/>
-    <tableColumn name="total_OpenMP_threads" id="10"/>
-    <tableColumn name="total_devices" id="11"/>
-    <tableColumn name="devices_per_node" id="12"/>
-    <tableColumn name="check" id="13"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="device"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="n_nodes"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="n_mpi_procs"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="n_omp_threads"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n_gpus"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="hpc_ensemble_partition"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="hpc_time_min_per_sim"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="total_OpenMP_threads"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="total_devices"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="devices_per_node"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="check"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -418,10 +433,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="44546A"/>
@@ -459,71 +474,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -551,7 +566,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -574,11 +589,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -587,13 +602,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -603,7 +618,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -612,7 +627,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -621,7 +636,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -629,10 +644,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -697,29 +712,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="22" width="29.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="22" width="9.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="23" width="9.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="24" width="19.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="24" width="22.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="24" width="28.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="24" width="28.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="25" width="28.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="24" width="28.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="24" width="24.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="24" width="19.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="24" width="19.862142857142857" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="25" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="29.85546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" style="21" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.28515625" style="22" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="28.28515625" style="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="28.28515625" style="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24.7109375" style="23" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.85546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -760,7 +774,7 @@
         <v>12</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row r="2" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>13</v>
       </c>
@@ -786,22 +800,27 @@
         <v>14</v>
       </c>
       <c r="I2" s="11">
-        <f>60*6</f>
+        <f t="shared" ref="I2:I41" si="0">60*6</f>
+        <v>360</v>
       </c>
       <c r="J2" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
       </c>
       <c r="K2" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
       </c>
       <c r="L2" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M2" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>13</v>
       </c>
@@ -827,22 +846,27 @@
         <v>14</v>
       </c>
       <c r="I3" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J3" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
       </c>
       <c r="K3" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>2</v>
       </c>
       <c r="L3" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M3" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+        <v>2</v>
+      </c>
+      <c r="M3" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>13</v>
       </c>
@@ -868,22 +892,27 @@
         <v>14</v>
       </c>
       <c r="I4" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J4" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>3</v>
       </c>
       <c r="K4" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>3</v>
       </c>
       <c r="L4" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M4" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+        <v>3</v>
+      </c>
+      <c r="M4" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>13</v>
       </c>
@@ -909,22 +938,27 @@
         <v>14</v>
       </c>
       <c r="I5" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J5" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
       </c>
       <c r="K5" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
       </c>
       <c r="L5" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M5" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+        <v>4</v>
+      </c>
+      <c r="M5" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>13</v>
       </c>
@@ -950,22 +984,27 @@
         <v>14</v>
       </c>
       <c r="I6" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J6" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>5</v>
       </c>
       <c r="K6" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>5</v>
       </c>
       <c r="L6" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M6" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+        <v>5</v>
+      </c>
+      <c r="M6" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>13</v>
       </c>
@@ -991,22 +1030,27 @@
         <v>14</v>
       </c>
       <c r="I7" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J7" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>6</v>
       </c>
       <c r="K7" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>6</v>
       </c>
       <c r="L7" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M7" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+        <v>6</v>
+      </c>
+      <c r="M7" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>13</v>
       </c>
@@ -1032,22 +1076,27 @@
         <v>14</v>
       </c>
       <c r="I8" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J8" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>7</v>
       </c>
       <c r="K8" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>7</v>
       </c>
       <c r="L8" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M8" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+        <v>7</v>
+      </c>
+      <c r="M8" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>13</v>
       </c>
@@ -1073,22 +1122,27 @@
         <v>14</v>
       </c>
       <c r="I9" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J9" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
       </c>
       <c r="K9" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
       </c>
       <c r="L9" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M9" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
+        <v>8</v>
+      </c>
+      <c r="M9" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>13</v>
       </c>
@@ -1114,26 +1168,31 @@
         <v>14</v>
       </c>
       <c r="I10" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J10" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K10" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
       </c>
       <c r="L10" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M10" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
-      <c r="A11" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="M10" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="10" t="s">
@@ -1155,38 +1214,43 @@
         <v>18</v>
       </c>
       <c r="I11" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J11" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
       </c>
       <c r="K11" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
       </c>
       <c r="L11" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M11" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
-      <c r="A12" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="M11" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="19">
         <v>1</v>
       </c>
       <c r="E12" s="11">
         <v>2</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="19">
         <v>4</v>
       </c>
       <c r="G12" s="11">
@@ -1196,26 +1260,31 @@
         <v>18</v>
       </c>
       <c r="I12" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J12" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
       </c>
       <c r="K12" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L12" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M12" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
-      <c r="A13" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="L12" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M12" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="10" t="s">
@@ -1237,26 +1306,31 @@
         <v>18</v>
       </c>
       <c r="I13" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J13" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
       </c>
       <c r="K13" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L13" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M13" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
-      <c r="A14" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="L13" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M13" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="10" t="s">
@@ -1278,26 +1352,31 @@
         <v>18</v>
       </c>
       <c r="I14" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J14" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K14" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L14" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M14" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
-      <c r="A15" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L14" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M14" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="10" t="s">
@@ -1319,26 +1398,31 @@
         <v>18</v>
       </c>
       <c r="I15" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J15" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K15" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L15" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M15" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
-      <c r="A16" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L15" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M15" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="10" t="s">
@@ -1360,26 +1444,31 @@
         <v>18</v>
       </c>
       <c r="I16" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J16" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K16" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L16" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M16" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
-      <c r="A17" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L16" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M16" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C17" s="10" t="s">
@@ -1401,26 +1490,31 @@
         <v>18</v>
       </c>
       <c r="I17" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J17" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
       </c>
       <c r="K17" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L17" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M17" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L17" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="M17" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="10" t="s">
@@ -1442,26 +1536,31 @@
         <v>18</v>
       </c>
       <c r="I18" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J18" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
       </c>
       <c r="K18" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L18" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M18" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L18" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="M18" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C19" s="10" t="s">
@@ -1483,26 +1582,31 @@
         <v>18</v>
       </c>
       <c r="I19" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J19" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
       </c>
       <c r="K19" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L19" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M19" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
-      <c r="A20" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L19" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="M19" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C20" s="10" t="s">
@@ -1524,26 +1628,31 @@
         <v>18</v>
       </c>
       <c r="I20" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J20" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
       </c>
       <c r="K20" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L20" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M20" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
-      <c r="A21" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L20" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="M20" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C21" s="10" t="s">
@@ -1565,26 +1674,31 @@
         <v>18</v>
       </c>
       <c r="I21" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J21" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K21" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L21" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M21" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
-      <c r="A22" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L21" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M21" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="10" t="s">
@@ -1606,26 +1720,31 @@
         <v>18</v>
       </c>
       <c r="I22" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J22" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K22" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L22" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M22" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
-      <c r="A23" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L22" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M22" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C23" s="10" t="s">
@@ -1647,26 +1766,31 @@
         <v>18</v>
       </c>
       <c r="I23" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J23" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K23" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L23" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M23" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
-      <c r="A24" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L23" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M23" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C24" s="10" t="s">
@@ -1688,26 +1812,31 @@
         <v>18</v>
       </c>
       <c r="I24" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J24" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K24" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L24" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M24" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
-      <c r="A25" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L24" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M24" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C25" s="10" t="s">
@@ -1729,26 +1858,31 @@
         <v>18</v>
       </c>
       <c r="I25" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J25" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K25" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L25" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M25" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
-      <c r="A26" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L25" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M25" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C26" s="10" t="s">
@@ -1770,26 +1904,31 @@
         <v>19</v>
       </c>
       <c r="I26" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J26" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K26" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L26" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M26" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
-      <c r="A27" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L26" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M26" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C27" s="10" t="s">
@@ -1811,26 +1950,31 @@
         <v>19</v>
       </c>
       <c r="I27" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J27" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K27" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L27" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M27" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
-      <c r="A28" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L27" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M27" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="10" t="s">
@@ -1852,26 +1996,31 @@
         <v>19</v>
       </c>
       <c r="I28" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J28" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K28" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L28" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M28" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
-      <c r="A29" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L28" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M28" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="10" t="s">
@@ -1893,26 +2042,31 @@
         <v>19</v>
       </c>
       <c r="I29" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J29" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K29" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L29" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M29" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
-      <c r="A30" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L29" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M29" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="10" t="s">
@@ -1934,26 +2088,31 @@
         <v>19</v>
       </c>
       <c r="I30" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J30" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K30" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L30" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M30" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L30" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M30" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C31" s="10" t="s">
@@ -1975,26 +2134,31 @@
         <v>19</v>
       </c>
       <c r="I31" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J31" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>128</v>
       </c>
       <c r="K31" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L31" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M31" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="L31" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M31" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C32" s="10" t="s">
@@ -2016,26 +2180,31 @@
         <v>18</v>
       </c>
       <c r="I32" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J32" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
       </c>
       <c r="K32" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L32" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M32" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="L32" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="M32" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="10" t="s">
@@ -2057,26 +2226,31 @@
         <v>18</v>
       </c>
       <c r="I33" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J33" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
       </c>
       <c r="K33" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L33" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M33" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="L33" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="M33" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C34" s="10" t="s">
@@ -2098,26 +2272,31 @@
         <v>18</v>
       </c>
       <c r="I34" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J34" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
       </c>
       <c r="K34" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L34" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M34" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="L34" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M34" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C35" s="10" t="s">
@@ -2139,26 +2318,31 @@
         <v>18</v>
       </c>
       <c r="I35" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J35" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K35" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L35" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M35" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L35" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M35" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B36" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C36" s="10" t="s">
@@ -2180,26 +2364,31 @@
         <v>18</v>
       </c>
       <c r="I36" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J36" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
       </c>
       <c r="K36" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L36" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M36" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="L36" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="M36" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C37" s="10" t="s">
@@ -2221,26 +2410,31 @@
         <v>18</v>
       </c>
       <c r="I37" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J37" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
       </c>
       <c r="K37" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L37" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M37" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="L37" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="M37" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B38" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C38" s="10" t="s">
@@ -2262,26 +2456,31 @@
         <v>18</v>
       </c>
       <c r="I38" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J38" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
       </c>
       <c r="K38" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L38" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M38" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="L38" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="M38" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="10" t="s">
@@ -2303,26 +2502,31 @@
         <v>18</v>
       </c>
       <c r="I39" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J39" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
       </c>
       <c r="K39" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L39" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M39" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="L39" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="M39" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C40" s="10" t="s">
@@ -2344,26 +2548,31 @@
         <v>18</v>
       </c>
       <c r="I40" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J40" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
       </c>
       <c r="K40" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L40" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M40" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="L40" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="M40" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C41" s="10" t="s">
@@ -2385,26 +2594,31 @@
         <v>18</v>
       </c>
       <c r="I41" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
+        <v>360</v>
       </c>
       <c r="J41" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
       </c>
       <c r="K41" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L41" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M41" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="L41" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="M41" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="B42" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C42" s="10" t="s">
@@ -2427,18 +2641,23 @@
       </c>
       <c r="I42" s="11">
         <f>60*12</f>
+        <v>720</v>
       </c>
       <c r="J42" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
       </c>
       <c r="K42" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-      </c>
-      <c r="L42" s="21">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-      </c>
-      <c r="M42" s="15">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="L42" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="M42" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change gpu partition to gpu-a6000
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1D0339-9B8D-4DF3-977A-B78BA3D86285}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B2503D-E221-4E11-BFD7-84B5E437B078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="27">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -111,6 +111,9 @@
   </si>
   <si>
     <t>serial</t>
+  </si>
+  <si>
+    <t>gpu-a6000</t>
   </si>
 </sst>
 </file>
@@ -797,7 +800,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I2" s="11">
         <f t="shared" ref="I2:I41" si="0">60*6</f>
@@ -843,7 +846,7 @@
         <v>2</v>
       </c>
       <c r="H3" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I3" s="11">
         <f t="shared" si="0"/>
@@ -889,7 +892,7 @@
         <v>3</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I4" s="11">
         <f t="shared" si="0"/>
@@ -935,7 +938,7 @@
         <v>4</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I5" s="11">
         <f t="shared" si="0"/>
@@ -981,7 +984,7 @@
         <v>5</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I6" s="11">
         <f t="shared" si="0"/>
@@ -1027,7 +1030,7 @@
         <v>6</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="0"/>
@@ -1073,7 +1076,7 @@
         <v>7</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I8" s="11">
         <f t="shared" si="0"/>
@@ -1119,7 +1122,7 @@
         <v>8</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I9" s="11">
         <f t="shared" si="0"/>
@@ -1165,7 +1168,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="I10" s="11">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
remove 32 mpi tests
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA71A68E-1EF3-4DF4-8B63-536DD66A2B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1962CA2-B976-44EA-87F0-C826B9B130C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="28">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -455,8 +455,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N42" totalsRowShown="0">
-  <autoFilter ref="A1:N42" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N39" totalsRowShown="0">
+  <autoFilter ref="A1:N39" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N39">
+    <sortCondition ref="C1:C39"/>
+  </sortState>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="device"/>
@@ -765,7 +768,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="21" bestFit="1" customWidth="1"/>
@@ -856,7 +859,7 @@
         <v>8</v>
       </c>
       <c r="J2" s="11">
-        <f t="shared" ref="J2:J41" si="0">60*6</f>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K2" s="13">
@@ -905,7 +908,7 @@
         <v>8</v>
       </c>
       <c r="J3" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K3" s="13">
@@ -954,7 +957,7 @@
         <v>8</v>
       </c>
       <c r="J4" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K4" s="13">
@@ -1003,7 +1006,7 @@
         <v>8</v>
       </c>
       <c r="J5" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K5" s="13">
@@ -1052,7 +1055,7 @@
         <v>8</v>
       </c>
       <c r="J6" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K6" s="13">
@@ -1101,7 +1104,7 @@
         <v>8</v>
       </c>
       <c r="J7" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K7" s="13">
@@ -1150,7 +1153,7 @@
         <v>8</v>
       </c>
       <c r="J8" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K8" s="13">
@@ -1199,7 +1202,7 @@
         <v>8</v>
       </c>
       <c r="J9" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K9" s="13">
@@ -1248,7 +1251,7 @@
         <v>8</v>
       </c>
       <c r="J10" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K10" s="13">
@@ -1297,7 +1300,7 @@
         <v>2</v>
       </c>
       <c r="J11" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K11" s="13">
@@ -1346,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="J12" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K12" s="13">
@@ -1395,7 +1398,7 @@
         <v>2</v>
       </c>
       <c r="J13" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K13" s="13">
@@ -1429,10 +1432,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G14" s="11">
         <v>0</v>
@@ -1444,7 +1447,7 @@
         <v>2</v>
       </c>
       <c r="J14" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K14" s="13">
@@ -1478,10 +1481,10 @@
         <v>1</v>
       </c>
       <c r="E15" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15" s="11">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G15" s="11">
         <v>0</v>
@@ -1493,7 +1496,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K15" s="13">
@@ -1542,7 +1545,7 @@
         <v>2</v>
       </c>
       <c r="J16" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K16" s="13">
@@ -1576,10 +1579,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F17" s="11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G17" s="11">
         <v>0</v>
@@ -1591,7 +1594,7 @@
         <v>2</v>
       </c>
       <c r="J17" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K17" s="13">
@@ -1625,10 +1628,10 @@
         <v>1</v>
       </c>
       <c r="E18" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G18" s="11">
         <v>0</v>
@@ -1640,7 +1643,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K18" s="13">
@@ -1674,10 +1677,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="11">
+        <v>8</v>
+      </c>
+      <c r="F19" s="11">
         <v>4</v>
-      </c>
-      <c r="F19" s="11">
-        <v>8</v>
       </c>
       <c r="G19" s="11">
         <v>0</v>
@@ -1689,7 +1692,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K19" s="13">
@@ -1723,10 +1726,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F20" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20" s="11">
         <v>0</v>
@@ -1738,7 +1741,7 @@
         <v>2</v>
       </c>
       <c r="J20" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K20" s="13">
@@ -1787,7 +1790,7 @@
         <v>2</v>
       </c>
       <c r="J21" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K21" s="13">
@@ -1821,10 +1824,10 @@
         <v>1</v>
       </c>
       <c r="E22" s="11">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="F22" s="11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G22" s="11">
         <v>0</v>
@@ -1836,7 +1839,7 @@
         <v>2</v>
       </c>
       <c r="J22" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K22" s="13">
@@ -1870,10 +1873,10 @@
         <v>1</v>
       </c>
       <c r="E23" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F23" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G23" s="11">
         <v>0</v>
@@ -1885,7 +1888,7 @@
         <v>2</v>
       </c>
       <c r="J23" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K23" s="13">
@@ -1934,7 +1937,7 @@
         <v>2</v>
       </c>
       <c r="J24" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K24" s="13">
@@ -1965,34 +1968,34 @@
         <v>17</v>
       </c>
       <c r="D25" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="11">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F25" s="11">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="G25" s="11">
         <v>0</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I25" s="12">
         <v>2</v>
       </c>
       <c r="J25" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K25" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="L25" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="M25" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -2017,10 +2020,10 @@
         <v>2</v>
       </c>
       <c r="E26" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F26" s="11">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="G26" s="11">
         <v>0</v>
@@ -2032,7 +2035,7 @@
         <v>2</v>
       </c>
       <c r="J26" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K26" s="13">
@@ -2066,10 +2069,10 @@
         <v>2</v>
       </c>
       <c r="E27" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F27" s="11">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G27" s="11">
         <v>0</v>
@@ -2081,7 +2084,7 @@
         <v>2</v>
       </c>
       <c r="J27" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K27" s="13">
@@ -2115,10 +2118,10 @@
         <v>2</v>
       </c>
       <c r="E28" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F28" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G28" s="11">
         <v>0</v>
@@ -2130,7 +2133,7 @@
         <v>2</v>
       </c>
       <c r="J28" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K28" s="13">
@@ -2152,47 +2155,47 @@
     </row>
     <row r="29" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B29" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D29" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F29" s="11">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G29" s="11">
         <v>0</v>
       </c>
       <c r="H29" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I29" s="12">
         <v>2</v>
       </c>
       <c r="J29" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K29" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="L29" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="M29" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N29" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2201,47 +2204,47 @@
     </row>
     <row r="30" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B30" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D30" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E30" s="11">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="F30" s="11">
+        <v>1</v>
+      </c>
+      <c r="G30" s="11">
+        <v>0</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="12">
+        <v>2</v>
+      </c>
+      <c r="J30" s="11">
+        <f>60*6</f>
+        <v>360</v>
+      </c>
+      <c r="K30" s="13">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="G30" s="11">
-        <v>0</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="I30" s="12">
-        <v>2</v>
-      </c>
-      <c r="J30" s="11">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="K30" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
-      </c>
       <c r="L30" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="M30" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="N30" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2250,47 +2253,47 @@
     </row>
     <row r="31" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B31" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D31" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="11">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F31" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="11">
         <v>0</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I31" s="12">
         <v>2</v>
       </c>
       <c r="J31" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K31" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="L31" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="M31" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N31" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2311,7 +2314,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="F32" s="11">
         <v>1</v>
@@ -2326,20 +2329,20 @@
         <v>2</v>
       </c>
       <c r="J32" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K32" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="L32" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="M32" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="N32" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2348,22 +2351,22 @@
     </row>
     <row r="33" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B33" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D33" s="11">
         <v>1</v>
       </c>
       <c r="E33" s="11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F33" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="11">
         <v>0</v>
@@ -2375,20 +2378,20 @@
         <v>2</v>
       </c>
       <c r="J33" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K33" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L33" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M33" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N33" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2397,22 +2400,22 @@
     </row>
     <row r="34" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B34" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D34" s="11">
         <v>1</v>
       </c>
       <c r="E34" s="11">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F34" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G34" s="11">
         <v>0</v>
@@ -2424,20 +2427,20 @@
         <v>2</v>
       </c>
       <c r="J34" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K34" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L34" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M34" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N34" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2446,22 +2449,22 @@
     </row>
     <row r="35" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B35" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D35" s="11">
         <v>1</v>
       </c>
       <c r="E35" s="11">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F35" s="11">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G35" s="11">
         <v>0</v>
@@ -2473,20 +2476,20 @@
         <v>2</v>
       </c>
       <c r="J35" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K35" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="L35" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="M35" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="N35" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2510,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="F36" s="11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G36" s="11">
         <v>0</v>
@@ -2522,20 +2525,20 @@
         <v>2</v>
       </c>
       <c r="J36" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K36" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="L36" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="M36" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="N36" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2559,7 +2562,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="11">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="G37" s="11">
         <v>0</v>
@@ -2571,20 +2574,20 @@
         <v>2</v>
       </c>
       <c r="J37" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K37" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="L37" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="M37" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="N37" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2608,7 +2611,7 @@
         <v>1</v>
       </c>
       <c r="F38" s="11">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="G38" s="11">
         <v>0</v>
@@ -2620,20 +2623,20 @@
         <v>2</v>
       </c>
       <c r="J38" s="11">
-        <f t="shared" si="0"/>
+        <f>60*6</f>
         <v>360</v>
       </c>
       <c r="K38" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="L38" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="M38" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="N38" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2642,13 +2645,13 @@
     </row>
     <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B39" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D39" s="11">
         <v>1</v>
@@ -2657,7 +2660,7 @@
         <v>1</v>
       </c>
       <c r="F39" s="11">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="G39" s="11">
         <v>0</v>
@@ -2669,169 +2672,22 @@
         <v>2</v>
       </c>
       <c r="J39" s="11">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="K39" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
-      </c>
-      <c r="L39" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="M39" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="N39" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C40" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D40" s="11">
-        <v>1</v>
-      </c>
-      <c r="E40" s="11">
-        <v>1</v>
-      </c>
-      <c r="F40" s="11">
-        <v>32</v>
-      </c>
-      <c r="G40" s="11">
-        <v>0</v>
-      </c>
-      <c r="H40" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I40" s="12">
-        <v>2</v>
-      </c>
-      <c r="J40" s="11">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="K40" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
-      </c>
-      <c r="L40" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
-      </c>
-      <c r="M40" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
-      </c>
-      <c r="N40" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="B41" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C41" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D41" s="11">
-        <v>1</v>
-      </c>
-      <c r="E41" s="11">
-        <v>1</v>
-      </c>
-      <c r="F41" s="11">
-        <v>64</v>
-      </c>
-      <c r="G41" s="11">
-        <v>0</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I41" s="12">
-        <v>2</v>
-      </c>
-      <c r="J41" s="11">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="K41" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
-      </c>
-      <c r="L41" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
-      </c>
-      <c r="M41" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
-      </c>
-      <c r="N41" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B42" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C42" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D42" s="11">
-        <v>1</v>
-      </c>
-      <c r="E42" s="11">
-        <v>1</v>
-      </c>
-      <c r="F42" s="11">
-        <v>1</v>
-      </c>
-      <c r="G42" s="11">
-        <v>0</v>
-      </c>
-      <c r="H42" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I42" s="12">
-        <v>2</v>
-      </c>
-      <c r="J42" s="11">
         <f>60*12</f>
         <v>720</v>
       </c>
-      <c r="K42" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
-      </c>
-      <c r="L42" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
-      </c>
-      <c r="M42" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-      <c r="N42" t="b">
+      <c r="K39" s="13">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="L39" s="13">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="M39" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="N39" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
remove 16 GPU test (we are very likely to hit diminishing returns with <8 GPUs which is the max with 16 removed)
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1962CA2-B976-44EA-87F0-C826B9B130C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B86984-E01B-467B-AE57-1EC3BB7D7310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="28">
   <si>
     <t>hardware_utilization_strategy</t>
   </si>
@@ -455,10 +455,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N39" totalsRowShown="0">
-  <autoFilter ref="A1:N39" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N39">
-    <sortCondition ref="C1:C39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:N38" totalsRowShown="0">
+  <autoFilter ref="A1:N38" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N38">
+    <sortCondition ref="C1:C38"/>
   </sortState>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="hardware_utilization_strategy"/>
@@ -768,7 +768,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" style="21" bestFit="1" customWidth="1"/>
@@ -859,7 +859,7 @@
         <v>8</v>
       </c>
       <c r="J2" s="11">
-        <f>60*6</f>
+        <f t="shared" ref="J2:J37" si="0">60*6</f>
         <v>360</v>
       </c>
       <c r="K2" s="13">
@@ -908,7 +908,7 @@
         <v>8</v>
       </c>
       <c r="J3" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K3" s="13">
@@ -957,7 +957,7 @@
         <v>8</v>
       </c>
       <c r="J4" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K4" s="13">
@@ -1006,7 +1006,7 @@
         <v>8</v>
       </c>
       <c r="J5" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K5" s="13">
@@ -1055,7 +1055,7 @@
         <v>8</v>
       </c>
       <c r="J6" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K6" s="13">
@@ -1104,7 +1104,7 @@
         <v>8</v>
       </c>
       <c r="J7" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K7" s="13">
@@ -1153,7 +1153,7 @@
         <v>8</v>
       </c>
       <c r="J8" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K8" s="13">
@@ -1202,7 +1202,7 @@
         <v>8</v>
       </c>
       <c r="J9" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K9" s="13">
@@ -1223,48 +1223,48 @@
       </c>
     </row>
     <row r="10" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>13</v>
+      <c r="A10" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>16</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E10" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F10" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" s="11">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="I10" s="12">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="J10" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K10" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="L10" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="M10" s="14">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N10" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1272,23 +1272,23 @@
       </c>
     </row>
     <row r="11" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="18" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="11">
+      <c r="D11" s="19">
         <v>1</v>
       </c>
       <c r="E11" s="11">
         <v>2</v>
       </c>
-      <c r="F11" s="11">
-        <v>2</v>
+      <c r="F11" s="19">
+        <v>4</v>
       </c>
       <c r="G11" s="11">
         <v>0</v>
@@ -1300,20 +1300,20 @@
         <v>2</v>
       </c>
       <c r="J11" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K11" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L11" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
-      </c>
-      <c r="M11" s="14">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="M11" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
       </c>
       <c r="N11" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1321,23 +1321,23 @@
       </c>
     </row>
     <row r="12" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="11">
         <v>1</v>
       </c>
       <c r="E12" s="11">
-        <v>2</v>
-      </c>
-      <c r="F12" s="19">
         <v>4</v>
+      </c>
+      <c r="F12" s="11">
+        <v>2</v>
       </c>
       <c r="G12" s="11">
         <v>0</v>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="J12" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K12" s="13">
@@ -1383,10 +1383,10 @@
         <v>1</v>
       </c>
       <c r="E13" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F13" s="11">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G13" s="11">
         <v>0</v>
@@ -1398,20 +1398,20 @@
         <v>2</v>
       </c>
       <c r="J13" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K13" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L13" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M13" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="N13" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1432,10 +1432,10 @@
         <v>1</v>
       </c>
       <c r="E14" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" s="11">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G14" s="11">
         <v>0</v>
@@ -1447,7 +1447,7 @@
         <v>2</v>
       </c>
       <c r="J14" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K14" s="13">
@@ -1481,10 +1481,10 @@
         <v>1</v>
       </c>
       <c r="E15" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F15" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G15" s="11">
         <v>0</v>
@@ -1496,7 +1496,7 @@
         <v>2</v>
       </c>
       <c r="J15" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K15" s="13">
@@ -1530,10 +1530,10 @@
         <v>1</v>
       </c>
       <c r="E16" s="11">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F16" s="11">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G16" s="11">
         <v>0</v>
@@ -1545,20 +1545,20 @@
         <v>2</v>
       </c>
       <c r="J16" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K16" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L16" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="M16" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="N16" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1579,10 +1579,10 @@
         <v>1</v>
       </c>
       <c r="E17" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F17" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G17" s="11">
         <v>0</v>
@@ -1594,7 +1594,7 @@
         <v>2</v>
       </c>
       <c r="J17" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K17" s="13">
@@ -1628,10 +1628,10 @@
         <v>1</v>
       </c>
       <c r="E18" s="11">
+        <v>8</v>
+      </c>
+      <c r="F18" s="11">
         <v>4</v>
-      </c>
-      <c r="F18" s="11">
-        <v>8</v>
       </c>
       <c r="G18" s="11">
         <v>0</v>
@@ -1643,7 +1643,7 @@
         <v>2</v>
       </c>
       <c r="J18" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K18" s="13">
@@ -1677,10 +1677,10 @@
         <v>1</v>
       </c>
       <c r="E19" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F19" s="11">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G19" s="11">
         <v>0</v>
@@ -1692,7 +1692,7 @@
         <v>2</v>
       </c>
       <c r="J19" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K19" s="13">
@@ -1726,10 +1726,10 @@
         <v>1</v>
       </c>
       <c r="E20" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F20" s="11">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="G20" s="11">
         <v>0</v>
@@ -1741,20 +1741,20 @@
         <v>2</v>
       </c>
       <c r="J20" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K20" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L20" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="M20" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="N20" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1775,10 +1775,10 @@
         <v>1</v>
       </c>
       <c r="E21" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F21" s="11">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G21" s="11">
         <v>0</v>
@@ -1790,7 +1790,7 @@
         <v>2</v>
       </c>
       <c r="J21" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K21" s="13">
@@ -1824,10 +1824,10 @@
         <v>1</v>
       </c>
       <c r="E22" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F22" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G22" s="11">
         <v>0</v>
@@ -1839,7 +1839,7 @@
         <v>2</v>
       </c>
       <c r="J22" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K22" s="13">
@@ -1873,10 +1873,10 @@
         <v>1</v>
       </c>
       <c r="E23" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F23" s="11">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G23" s="11">
         <v>0</v>
@@ -1888,7 +1888,7 @@
         <v>2</v>
       </c>
       <c r="J23" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K23" s="13">
@@ -1919,34 +1919,34 @@
         <v>17</v>
       </c>
       <c r="D24" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F24" s="11">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="G24" s="11">
         <v>0</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I24" s="12">
         <v>2</v>
       </c>
       <c r="J24" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K24" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="L24" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="M24" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1971,10 +1971,10 @@
         <v>2</v>
       </c>
       <c r="E25" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F25" s="11">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="G25" s="11">
         <v>0</v>
@@ -1986,7 +1986,7 @@
         <v>2</v>
       </c>
       <c r="J25" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K25" s="13">
@@ -2020,10 +2020,10 @@
         <v>2</v>
       </c>
       <c r="E26" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F26" s="11">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G26" s="11">
         <v>0</v>
@@ -2035,7 +2035,7 @@
         <v>2</v>
       </c>
       <c r="J26" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K26" s="13">
@@ -2069,10 +2069,10 @@
         <v>2</v>
       </c>
       <c r="E27" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F27" s="11">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="G27" s="11">
         <v>0</v>
@@ -2084,7 +2084,7 @@
         <v>2</v>
       </c>
       <c r="J27" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K27" s="13">
@@ -2106,47 +2106,47 @@
     </row>
     <row r="28" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D28" s="11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="11">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F28" s="11">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G28" s="11">
         <v>0</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I28" s="12">
         <v>2</v>
       </c>
       <c r="J28" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K28" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="L28" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="M28" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="N28" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2167,7 +2167,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F29" s="11">
         <v>1</v>
@@ -2182,27 +2182,27 @@
         <v>2</v>
       </c>
       <c r="J29" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K29" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L29" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M29" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N29" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
         <v>20</v>
       </c>
@@ -2216,7 +2216,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F30" s="11">
         <v>1</v>
@@ -2231,20 +2231,20 @@
         <v>2</v>
       </c>
       <c r="J30" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K30" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L30" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M30" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N30" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2265,7 +2265,7 @@
         <v>1</v>
       </c>
       <c r="E31" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F31" s="11">
         <v>1</v>
@@ -2280,20 +2280,20 @@
         <v>2</v>
       </c>
       <c r="J31" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K31" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L31" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M31" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="N31" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2302,22 +2302,22 @@
     </row>
     <row r="32" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D32" s="11">
         <v>1</v>
       </c>
       <c r="E32" s="11">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F32" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="11">
         <v>0</v>
@@ -2329,20 +2329,20 @@
         <v>2</v>
       </c>
       <c r="J32" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K32" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="L32" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="M32" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="N32" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2366,7 +2366,7 @@
         <v>1</v>
       </c>
       <c r="F33" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G33" s="11">
         <v>0</v>
@@ -2378,20 +2378,20 @@
         <v>2</v>
       </c>
       <c r="J33" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K33" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L33" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M33" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N33" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2415,7 +2415,7 @@
         <v>1</v>
       </c>
       <c r="F34" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G34" s="11">
         <v>0</v>
@@ -2427,20 +2427,20 @@
         <v>2</v>
       </c>
       <c r="J34" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K34" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L34" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M34" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="N34" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2464,7 +2464,7 @@
         <v>1</v>
       </c>
       <c r="F35" s="11">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G35" s="11">
         <v>0</v>
@@ -2476,20 +2476,20 @@
         <v>2</v>
       </c>
       <c r="J35" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K35" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L35" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="M35" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="N35" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2513,7 +2513,7 @@
         <v>1</v>
       </c>
       <c r="F36" s="11">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G36" s="11">
         <v>0</v>
@@ -2525,20 +2525,20 @@
         <v>2</v>
       </c>
       <c r="J36" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K36" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L36" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="M36" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="N36" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2562,7 +2562,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="11">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="G37" s="11">
         <v>0</v>
@@ -2574,20 +2574,20 @@
         <v>2</v>
       </c>
       <c r="J37" s="11">
-        <f>60*6</f>
+        <f t="shared" si="0"/>
         <v>360</v>
       </c>
       <c r="K37" s="13">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L37" s="13">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="M37" s="20">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="N37" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2596,13 +2596,13 @@
     </row>
     <row r="38" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B38" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D38" s="11">
         <v>1</v>
@@ -2611,7 +2611,7 @@
         <v>1</v>
       </c>
       <c r="F38" s="11">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="G38" s="11">
         <v>0</v>
@@ -2623,71 +2623,22 @@
         <v>2</v>
       </c>
       <c r="J38" s="11">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="K38" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
-      </c>
-      <c r="L38" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
-      </c>
-      <c r="M38" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
-      </c>
-      <c r="N38" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="B39" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C39" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D39" s="11">
-        <v>1</v>
-      </c>
-      <c r="E39" s="11">
-        <v>1</v>
-      </c>
-      <c r="F39" s="11">
-        <v>1</v>
-      </c>
-      <c r="G39" s="11">
-        <v>0</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="I39" s="12">
-        <v>2</v>
-      </c>
-      <c r="J39" s="11">
         <f>60*12</f>
         <v>720</v>
       </c>
-      <c r="K39" s="13">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
-      </c>
-      <c r="L39" s="13">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
-      </c>
-      <c r="M39" s="20">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-      <c r="N39" t="b">
+      <c r="K38" s="13">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="L38" s="13">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="M38" s="20">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="N38" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
remove >2 GPU runs and add 2 a100 runs
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DFDE6D-F952-402E-A8FF-73FEFCC3D08F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE66675C-6A7B-4760-812B-7827FD9F159D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="4185" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="21">
   <si>
     <t>run_mode</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>mem_gb_per_cpu</t>
+  </si>
+  <si>
+    <t>gpu-a100</t>
   </si>
 </sst>
 </file>
@@ -361,10 +364,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L38" totalsRowShown="0">
-  <autoFilter ref="A1:L38" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L38">
-    <sortCondition ref="A1:A38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L34" totalsRowShown="0">
+  <autoFilter ref="A1:L34" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L34">
+    <sortCondition ref="A1:A34"/>
   </sortState>
   <tableColumns count="12">
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
@@ -672,7 +675,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="14" bestFit="1" customWidth="1"/>
@@ -749,7 +752,7 @@
         <v>8</v>
       </c>
       <c r="H2" s="8">
-        <f t="shared" ref="H2:H37" si="0">60*6</f>
+        <f t="shared" ref="H2:H33" si="0">60*6</f>
         <v>360</v>
       </c>
       <c r="I2" s="10">
@@ -826,10 +829,10 @@
         <v>1</v>
       </c>
       <c r="E4" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G4" s="9">
         <v>8</v>
@@ -869,10 +872,10 @@
         <v>1</v>
       </c>
       <c r="E5" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G5" s="9">
         <v>8</v>
@@ -900,25 +903,25 @@
     </row>
     <row r="6" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="8">
         <v>1</v>
       </c>
       <c r="C6" s="8">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D6" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G6" s="9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H6" s="8">
         <f t="shared" si="0"/>
@@ -926,15 +929,15 @@
       </c>
       <c r="I6" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J6" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6" s="11">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L6" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -943,25 +946,25 @@
     </row>
     <row r="7" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="8">
+        <v>12</v>
+      </c>
+      <c r="B7" s="12">
         <v>1</v>
       </c>
       <c r="C7" s="8">
-        <v>6</v>
-      </c>
-      <c r="D7" s="8">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D7" s="12">
+        <v>4</v>
       </c>
       <c r="E7" s="8">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G7" s="9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H7" s="8">
         <f t="shared" si="0"/>
@@ -969,15 +972,15 @@
       </c>
       <c r="I7" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J7" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>6</v>
-      </c>
-      <c r="K7" s="11">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="K7" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
       </c>
       <c r="L7" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -986,25 +989,25 @@
     </row>
     <row r="8" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="8">
         <v>1</v>
       </c>
       <c r="C8" s="8">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8" s="8">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G8" s="9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H8" s="8">
         <f t="shared" si="0"/>
@@ -1012,15 +1015,15 @@
       </c>
       <c r="I8" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>7</v>
-      </c>
-      <c r="K8" s="11">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="K8" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
       </c>
       <c r="L8" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1029,25 +1032,25 @@
     </row>
     <row r="9" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="8">
         <v>1</v>
       </c>
       <c r="C9" s="8">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D9" s="8">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E9" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G9" s="9">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H9" s="8">
         <f t="shared" si="0"/>
@@ -1055,15 +1058,15 @@
       </c>
       <c r="I9" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J9" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K9" s="11">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>16</v>
+      </c>
+      <c r="K9" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
       </c>
       <c r="L9" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1078,10 +1081,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D10" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E10" s="8">
         <v>0</v>
@@ -1098,15 +1101,15 @@
       </c>
       <c r="I10" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J10" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
-      </c>
-      <c r="K10" s="11">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>16</v>
+      </c>
+      <c r="K10" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
       </c>
       <c r="L10" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1117,14 +1120,14 @@
       <c r="A11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="8">
         <v>1</v>
       </c>
       <c r="C11" s="8">
-        <v>2</v>
-      </c>
-      <c r="D11" s="12">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="D11" s="8">
+        <v>2</v>
       </c>
       <c r="E11" s="8">
         <v>0</v>
@@ -1141,15 +1144,15 @@
       </c>
       <c r="I11" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="J11" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="K11" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="L11" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1164,10 +1167,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D12" s="8">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E12" s="8">
         <v>0</v>
@@ -1184,15 +1187,15 @@
       </c>
       <c r="I12" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="J12" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="K12" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="L12" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1207,7 +1210,7 @@
         <v>1</v>
       </c>
       <c r="C13" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D13" s="8">
         <v>8</v>
@@ -1227,15 +1230,15 @@
       </c>
       <c r="I13" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J13" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="K13" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L13" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1250,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="C14" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D14" s="8">
         <v>4</v>
@@ -1270,15 +1273,15 @@
       </c>
       <c r="I14" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J14" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="K14" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L14" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1293,7 +1296,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="8">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D15" s="8">
         <v>2</v>
@@ -1313,15 +1316,15 @@
       </c>
       <c r="I15" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="J15" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="K15" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L15" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1339,7 +1342,7 @@
         <v>2</v>
       </c>
       <c r="D16" s="8">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E16" s="8">
         <v>0</v>
@@ -1356,15 +1359,15 @@
       </c>
       <c r="I16" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="J16" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="K16" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L16" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1382,7 +1385,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="8">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E17" s="8">
         <v>0</v>
@@ -1399,15 +1402,15 @@
       </c>
       <c r="I17" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="J17" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="K17" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L17" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1425,7 +1428,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E18" s="8">
         <v>0</v>
@@ -1442,15 +1445,15 @@
       </c>
       <c r="I18" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="J18" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="K18" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L18" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1468,7 +1471,7 @@
         <v>16</v>
       </c>
       <c r="D19" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E19" s="8">
         <v>0</v>
@@ -1485,15 +1488,15 @@
       </c>
       <c r="I19" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="J19" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="K19" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="L19" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1505,19 +1508,19 @@
         <v>12</v>
       </c>
       <c r="B20" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C20" s="8">
         <v>2</v>
       </c>
       <c r="D20" s="8">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="E20" s="8">
         <v>0</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G20" s="9">
         <v>2</v>
@@ -1528,11 +1531,11 @@
       </c>
       <c r="I20" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="J20" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="K20" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1548,19 +1551,19 @@
         <v>12</v>
       </c>
       <c r="B21" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C21" s="8">
         <v>4</v>
       </c>
       <c r="D21" s="8">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E21" s="8">
         <v>0</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G21" s="9">
         <v>2</v>
@@ -1571,11 +1574,11 @@
       </c>
       <c r="I21" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="J21" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="K21" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1591,19 +1594,19 @@
         <v>12</v>
       </c>
       <c r="B22" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C22" s="8">
         <v>8</v>
       </c>
       <c r="D22" s="8">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E22" s="8">
         <v>0</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G22" s="9">
         <v>2</v>
@@ -1614,11 +1617,11 @@
       </c>
       <c r="I22" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="J22" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="K22" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1634,19 +1637,19 @@
         <v>12</v>
       </c>
       <c r="B23" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" s="8">
         <v>16</v>
       </c>
       <c r="D23" s="8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E23" s="8">
         <v>0</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G23" s="9">
         <v>2</v>
@@ -1657,11 +1660,11 @@
       </c>
       <c r="I23" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="J23" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="K23" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1674,22 +1677,22 @@
     </row>
     <row r="24" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B24" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24" s="8">
         <v>2</v>
       </c>
       <c r="D24" s="8">
-        <v>64</v>
+        <v>1</v>
       </c>
       <c r="E24" s="8">
         <v>0</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G24" s="9">
         <v>2</v>
@@ -1700,15 +1703,15 @@
       </c>
       <c r="I24" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="J24" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>2</v>
       </c>
       <c r="K24" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="L24" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1717,22 +1720,22 @@
     </row>
     <row r="25" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B25" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" s="8">
         <v>4</v>
       </c>
       <c r="D25" s="8">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E25" s="8">
         <v>0</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G25" s="9">
         <v>2</v>
@@ -1743,39 +1746,39 @@
       </c>
       <c r="I25" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="J25" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>4</v>
       </c>
       <c r="K25" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="L25" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B26" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" s="8">
         <v>8</v>
       </c>
       <c r="D26" s="8">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E26" s="8">
         <v>0</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G26" s="9">
         <v>2</v>
@@ -1786,39 +1789,39 @@
       </c>
       <c r="I26" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="J26" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>8</v>
       </c>
       <c r="K26" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L26" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B27" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="8">
         <v>16</v>
       </c>
       <c r="D27" s="8">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E27" s="8">
         <v>0</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G27" s="9">
         <v>2</v>
@@ -1829,33 +1832,33 @@
       </c>
       <c r="I27" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="J27" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>16</v>
       </c>
       <c r="K27" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="L27" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B28" s="8">
         <v>1</v>
       </c>
       <c r="C28" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D28" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E28" s="8">
         <v>0</v>
@@ -1887,18 +1890,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B29" s="8">
         <v>1</v>
       </c>
       <c r="C29" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D29" s="8">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E29" s="8">
         <v>0</v>
@@ -1932,16 +1935,16 @@
     </row>
     <row r="30" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B30" s="8">
         <v>1</v>
       </c>
       <c r="C30" s="8">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D30" s="8">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E30" s="8">
         <v>0</v>
@@ -1975,16 +1978,16 @@
     </row>
     <row r="31" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B31" s="8">
         <v>1</v>
       </c>
       <c r="C31" s="8">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="D31" s="8">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E31" s="8">
         <v>0</v>
@@ -2027,7 +2030,7 @@
         <v>1</v>
       </c>
       <c r="D32" s="8">
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="E32" s="8">
         <v>0</v>
@@ -2044,15 +2047,15 @@
       </c>
       <c r="I32" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="J32" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="K32" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>32</v>
       </c>
       <c r="L32" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2070,7 +2073,7 @@
         <v>1</v>
       </c>
       <c r="D33" s="8">
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="E33" s="8">
         <v>0</v>
@@ -2087,15 +2090,15 @@
       </c>
       <c r="I33" s="10">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="J33" s="10">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="K33" s="13">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>64</v>
       </c>
       <c r="L33" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -2104,7 +2107,7 @@
     </row>
     <row r="34" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B34" s="8">
         <v>1</v>
@@ -2113,7 +2116,7 @@
         <v>1</v>
       </c>
       <c r="D34" s="8">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E34" s="8">
         <v>0</v>
@@ -2125,194 +2128,22 @@
         <v>2</v>
       </c>
       <c r="H34" s="8">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="I34" s="10">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
-      </c>
-      <c r="J34" s="10">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
-      </c>
-      <c r="K34" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
-      </c>
-      <c r="L34" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B35" s="8">
-        <v>1</v>
-      </c>
-      <c r="C35" s="8">
-        <v>1</v>
-      </c>
-      <c r="D35" s="8">
-        <v>16</v>
-      </c>
-      <c r="E35" s="8">
-        <v>0</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G35" s="9">
-        <v>2</v>
-      </c>
-      <c r="H35" s="8">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="I35" s="10">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
-      </c>
-      <c r="J35" s="10">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
-      </c>
-      <c r="K35" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
-      </c>
-      <c r="L35" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B36" s="8">
-        <v>1</v>
-      </c>
-      <c r="C36" s="8">
-        <v>1</v>
-      </c>
-      <c r="D36" s="8">
-        <v>32</v>
-      </c>
-      <c r="E36" s="8">
-        <v>0</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G36" s="9">
-        <v>2</v>
-      </c>
-      <c r="H36" s="8">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="I36" s="10">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
-      </c>
-      <c r="J36" s="10">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
-      </c>
-      <c r="K36" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
-      </c>
-      <c r="L36" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B37" s="8">
-        <v>1</v>
-      </c>
-      <c r="C37" s="8">
-        <v>1</v>
-      </c>
-      <c r="D37" s="8">
-        <v>64</v>
-      </c>
-      <c r="E37" s="8">
-        <v>0</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G37" s="9">
-        <v>2</v>
-      </c>
-      <c r="H37" s="8">
-        <f t="shared" si="0"/>
-        <v>360</v>
-      </c>
-      <c r="I37" s="10">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
-      </c>
-      <c r="J37" s="10">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
-      </c>
-      <c r="K37" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
-      </c>
-      <c r="L37" t="b">
-        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B38" s="8">
-        <v>1</v>
-      </c>
-      <c r="C38" s="8">
-        <v>1</v>
-      </c>
-      <c r="D38" s="8">
-        <v>1</v>
-      </c>
-      <c r="E38" s="8">
-        <v>0</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="9">
-        <v>2</v>
-      </c>
-      <c r="H38" s="8">
         <f>60*12</f>
         <v>720</v>
       </c>
-      <c r="I38" s="10">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
-      </c>
-      <c r="J38" s="10">
-        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
-      </c>
-      <c r="K38" s="13">
-        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
-      </c>
-      <c r="L38" t="b">
+      <c r="I34" s="10">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="J34" s="10">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="K34" s="13">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="L34" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
data: remove sa_33 row from UVA sensitivity XLSX (Phase 6 Stage 3 Part D — remove-scenario smoke verification)
Removes the sa_33 row added in commit e868653 for Part C add-scenario
smoke testing. Part D verifies the inverse workflow: user removes a
sub-analysis from the XLSX, pushes, pulls on Rivanna, runs analysis.run()
— and snakemake should plan zero new work (sa_33's outputs already
satisfy nothing; sa_33 is no longer in the sensitivity definition).

Companion to commit 2b30a47 (sa_2/sa_3 removal). Final post-edit state:
sa_0, sa_1, sa_4..sa_32 = 31 sub-analyses; sa_33 was the temporary smoke
target only.

XLSX shape after edit: 31 rows; hpc_time_min_per_sim populated for all
rows (sa_0..sa_31 = 360, sa_32 = 720).
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="21">
   <si>
     <t xml:space="preserve">sa_id</t>
   </si>
@@ -172,7 +172,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -183,10 +183,6 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1339,35 +1335,7 @@
         <v>720</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="n">
-        <v>33</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E33" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H33" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="I33" s="1" t="n">
-        <v>360</v>
-      </c>
-    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>